<commit_message>
Aggiornato giacenza.xlsx da lbianco via Streamlit
</commit_message>
<xml_diff>
--- a/giacenza.xlsx
+++ b/giacenza.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1301" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1332" uniqueCount="24">
   <si>
     <t>Data</t>
   </si>
@@ -821,14 +821,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U1299"/>
+  <dimension ref="A1:U1330"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.85546875" customWidth="1"/>
     <col min="2" max="2" width="25.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="22.28515625" customWidth="1"/>
+    <col min="6" max="6" width="22.42578125" customWidth="1"/>
     <col min="7" max="9" width="29.42578125" customWidth="1"/>
     <col min="10" max="11" width="22.7109375" customWidth="1"/>
     <col min="12" max="12" width="22.7109375" bestFit="1" customWidth="1"/>
@@ -20603,7 +20603,9 @@
       <c r="C1290" s="6">
         <v>2</v>
       </c>
-      <c r="D1290" s="2"/>
+      <c r="D1290" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1291" spans="1:7">
       <c r="A1291" s="7">
@@ -20615,7 +20617,9 @@
       <c r="C1291" s="6">
         <v>2</v>
       </c>
-      <c r="D1291" s="2"/>
+      <c r="D1291" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1292" spans="1:7">
       <c r="A1292" s="7">
@@ -20627,7 +20631,9 @@
       <c r="C1292" s="6">
         <v>5</v>
       </c>
-      <c r="D1292" s="2"/>
+      <c r="D1292" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="1293" spans="1:7">
       <c r="A1293" s="7">
@@ -20639,7 +20645,9 @@
       <c r="C1293" s="6">
         <v>5</v>
       </c>
-      <c r="D1293" s="2"/>
+      <c r="D1293" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="1294" spans="1:7">
       <c r="A1294" s="7">
@@ -20651,7 +20659,9 @@
       <c r="C1294" s="6">
         <v>3</v>
       </c>
-      <c r="D1294" s="2"/>
+      <c r="D1294" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1295" spans="1:7">
       <c r="A1295" s="7">
@@ -20663,7 +20673,9 @@
       <c r="C1295" s="6">
         <v>3</v>
       </c>
-      <c r="D1295" s="2"/>
+      <c r="D1295" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1296" spans="1:7">
       <c r="A1296" s="7">
@@ -20675,9 +20687,11 @@
       <c r="C1296" s="6">
         <v>2</v>
       </c>
-      <c r="D1296" s="2"/>
-    </row>
-    <row r="1297" spans="1:4">
+      <c r="D1296" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1297" spans="1:7">
       <c r="A1297" s="7">
         <v>46077</v>
       </c>
@@ -20687,31 +20701,483 @@
       <c r="C1297" s="6">
         <v>2</v>
       </c>
-      <c r="D1297" s="2"/>
-    </row>
-    <row r="1298" spans="1:4">
+      <c r="D1297" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1298" spans="1:7">
       <c r="A1298" s="7">
         <v>46077</v>
       </c>
-      <c r="B1298" s="2" t="s">
+      <c r="B1298" s="70" t="s">
         <v>23</v>
       </c>
       <c r="C1298" s="6">
         <v>5</v>
       </c>
-      <c r="D1298" s="2"/>
-    </row>
-    <row r="1299" spans="1:4">
+      <c r="D1298" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1299" spans="1:7">
       <c r="A1299" s="7">
         <v>46077</v>
       </c>
-      <c r="B1299" s="2" t="s">
+      <c r="B1299" s="70" t="s">
         <v>21</v>
       </c>
       <c r="C1299" s="2">
         <v>5</v>
       </c>
-      <c r="D1299" s="2"/>
+      <c r="D1299" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1300" spans="1:7">
+      <c r="A1300" s="7">
+        <v>46077</v>
+      </c>
+      <c r="B1300" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1300" s="6">
+        <v>0</v>
+      </c>
+      <c r="D1300" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1301" spans="1:7">
+      <c r="A1301" s="7">
+        <v>46078</v>
+      </c>
+      <c r="B1301" s="66" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1301" s="6">
+        <v>4</v>
+      </c>
+      <c r="D1301" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1301" s="1"/>
+      <c r="G1301" s="22"/>
+    </row>
+    <row r="1302" spans="1:7">
+      <c r="A1302" s="7">
+        <v>46078</v>
+      </c>
+      <c r="B1302" s="66" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1302" s="6">
+        <v>4</v>
+      </c>
+      <c r="D1302" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1302" s="1"/>
+      <c r="G1302" s="22"/>
+    </row>
+    <row r="1303" spans="1:7">
+      <c r="A1303" s="7">
+        <v>46078</v>
+      </c>
+      <c r="B1303" s="56" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1303" s="6">
+        <v>2</v>
+      </c>
+      <c r="D1303" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1303" s="1"/>
+      <c r="G1303" s="22"/>
+    </row>
+    <row r="1304" spans="1:7">
+      <c r="A1304" s="7">
+        <v>46078</v>
+      </c>
+      <c r="B1304" s="56" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1304" s="6">
+        <v>2</v>
+      </c>
+      <c r="D1304" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1304" s="1"/>
+      <c r="G1304" s="22"/>
+    </row>
+    <row r="1305" spans="1:7">
+      <c r="A1305" s="7">
+        <v>46078</v>
+      </c>
+      <c r="B1305" s="57" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1305" s="6">
+        <v>2</v>
+      </c>
+      <c r="D1305" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1305" s="1"/>
+      <c r="G1305" s="22"/>
+    </row>
+    <row r="1306" spans="1:7">
+      <c r="A1306" s="7">
+        <v>46078</v>
+      </c>
+      <c r="B1306" s="57" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1306" s="6">
+        <v>2</v>
+      </c>
+      <c r="D1306" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1306" s="1"/>
+      <c r="G1306" s="22"/>
+    </row>
+    <row r="1307" spans="1:7">
+      <c r="A1307" s="7">
+        <v>46078</v>
+      </c>
+      <c r="B1307" s="59" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1307" s="6">
+        <v>1</v>
+      </c>
+      <c r="D1307" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1307" s="1"/>
+      <c r="G1307" s="22"/>
+    </row>
+    <row r="1308" spans="1:7">
+      <c r="A1308" s="7">
+        <v>46078</v>
+      </c>
+      <c r="B1308" s="59" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1308" s="2">
+        <v>1</v>
+      </c>
+      <c r="D1308" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1308" s="1"/>
+      <c r="G1308" s="22"/>
+    </row>
+    <row r="1309" spans="1:7">
+      <c r="A1309" s="7">
+        <v>46078</v>
+      </c>
+      <c r="B1309" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1309" s="2">
+        <v>8</v>
+      </c>
+      <c r="D1309" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1310" spans="1:7">
+      <c r="A1310" s="7">
+        <v>46078</v>
+      </c>
+      <c r="B1310" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1310" s="2">
+        <v>0</v>
+      </c>
+      <c r="D1310" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1311" spans="1:7">
+      <c r="A1311" s="7">
+        <v>46078</v>
+      </c>
+      <c r="B1311" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1311" s="2">
+        <v>0</v>
+      </c>
+      <c r="D1311" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1312" spans="1:7">
+      <c r="A1312" s="7">
+        <v>46078</v>
+      </c>
+      <c r="B1312" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1312" s="2">
+        <v>0</v>
+      </c>
+      <c r="D1312" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1313" spans="1:7">
+      <c r="A1313" s="7">
+        <v>46079</v>
+      </c>
+      <c r="B1313" s="70" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1313" s="2">
+        <v>0</v>
+      </c>
+      <c r="D1313" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1314" spans="1:7">
+      <c r="A1314" s="7">
+        <v>46079</v>
+      </c>
+      <c r="B1314" s="70" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1314" s="2">
+        <v>0</v>
+      </c>
+      <c r="D1314" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1315" spans="1:7">
+      <c r="A1315" s="7">
+        <v>46079</v>
+      </c>
+      <c r="B1315" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1315" s="6">
+        <v>6</v>
+      </c>
+      <c r="D1315" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1316" spans="1:7">
+      <c r="A1316" s="7">
+        <v>46079</v>
+      </c>
+      <c r="B1316" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1316" s="6">
+        <v>6</v>
+      </c>
+      <c r="D1316" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1316" s="1"/>
+      <c r="G1316" s="22"/>
+    </row>
+    <row r="1317" spans="1:7">
+      <c r="A1317" s="7">
+        <v>46079</v>
+      </c>
+      <c r="B1317" s="64" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1317" s="6">
+        <v>1</v>
+      </c>
+      <c r="D1317" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1317" s="1"/>
+      <c r="G1317" s="22"/>
+    </row>
+    <row r="1318" spans="1:7">
+      <c r="A1318" s="7">
+        <v>46079</v>
+      </c>
+      <c r="B1318" s="64" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1318" s="6">
+        <v>1</v>
+      </c>
+      <c r="D1318" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1318" s="1"/>
+      <c r="G1318" s="22"/>
+    </row>
+    <row r="1319" spans="1:7">
+      <c r="A1319" s="7">
+        <v>46079</v>
+      </c>
+      <c r="B1319" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1319" s="6">
+        <v>4</v>
+      </c>
+      <c r="D1319" s="2">
+        <v>9</v>
+      </c>
+      <c r="F1319" s="1"/>
+      <c r="G1319" s="22"/>
+    </row>
+    <row r="1320" spans="1:7">
+      <c r="A1320" s="7">
+        <v>46079</v>
+      </c>
+      <c r="B1320" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1320" s="6">
+        <v>4</v>
+      </c>
+      <c r="D1320" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1320" s="1"/>
+      <c r="G1320" s="22"/>
+    </row>
+    <row r="1321" spans="1:7">
+      <c r="A1321" s="7">
+        <v>46080</v>
+      </c>
+      <c r="B1321" s="64" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1321" s="6">
+        <v>3</v>
+      </c>
+      <c r="D1321" s="2"/>
+      <c r="F1321" s="1"/>
+      <c r="G1321" s="22"/>
+    </row>
+    <row r="1322" spans="1:7">
+      <c r="A1322" s="7">
+        <v>46080</v>
+      </c>
+      <c r="B1322" s="64" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1322" s="6">
+        <v>3</v>
+      </c>
+      <c r="D1322" s="2"/>
+      <c r="F1322" s="1"/>
+      <c r="G1322" s="22"/>
+    </row>
+    <row r="1323" spans="1:7">
+      <c r="A1323" s="7">
+        <v>46080</v>
+      </c>
+      <c r="B1323" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1323" s="6">
+        <v>9</v>
+      </c>
+      <c r="D1323" s="2"/>
+      <c r="F1323" s="1"/>
+      <c r="G1323" s="22"/>
+    </row>
+    <row r="1324" spans="1:7">
+      <c r="A1324" s="7">
+        <v>46080</v>
+      </c>
+      <c r="B1324" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1324" s="6">
+        <v>9</v>
+      </c>
+      <c r="D1324" s="2"/>
+    </row>
+    <row r="1325" spans="1:7">
+      <c r="A1325" s="7">
+        <v>46080</v>
+      </c>
+      <c r="B1325" s="56" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1325" s="6">
+        <v>5</v>
+      </c>
+      <c r="D1325" s="2"/>
+    </row>
+    <row r="1326" spans="1:7">
+      <c r="A1326" s="7">
+        <v>46080</v>
+      </c>
+      <c r="B1326" s="56" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1326" s="6">
+        <v>5</v>
+      </c>
+      <c r="D1326" s="2"/>
+    </row>
+    <row r="1327" spans="1:7">
+      <c r="A1327" s="7">
+        <v>46080</v>
+      </c>
+      <c r="B1327" s="57" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1327" s="6">
+        <v>5</v>
+      </c>
+      <c r="D1327" s="2"/>
+    </row>
+    <row r="1328" spans="1:7">
+      <c r="A1328" s="7">
+        <v>46080</v>
+      </c>
+      <c r="B1328" s="57" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1328" s="6">
+        <v>5</v>
+      </c>
+      <c r="D1328" s="2"/>
+    </row>
+    <row r="1329" spans="1:4">
+      <c r="A1329" s="7">
+        <v>46080</v>
+      </c>
+      <c r="B1329" s="59" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1329" s="6">
+        <v>7</v>
+      </c>
+      <c r="D1329" s="2"/>
+    </row>
+    <row r="1330" spans="1:4">
+      <c r="A1330" s="7">
+        <v>46080</v>
+      </c>
+      <c r="B1330" s="59" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1330" s="6">
+        <v>7</v>
+      </c>
+      <c r="D1330" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D106"/>

</xml_diff>